<commit_message>
feat: material-weighted procurement forecast and UI/workflow updates
</commit_message>
<xml_diff>
--- a/materials.xlsx
+++ b/materials.xlsx
@@ -7,8 +7,9 @@
     <sheet name="Запасы" sheetId="2" r:id="rId2"/>
     <sheet name="Min" sheetId="3" r:id="rId3"/>
     <sheet name="Прогноз_продаж" sheetId="4" r:id="rId4"/>
-    <sheet name="Прогноз_закупок" sheetId="5" r:id="rId5"/>
-    <sheet name="Методы" sheetId="6" r:id="rId6"/>
+    <sheet name="Закупки" sheetId="5" r:id="rId5"/>
+    <sheet name="Прогноз_закупок" sheetId="6" r:id="rId6"/>
+    <sheet name="Методы" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -7872,6 +7873,135 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>CW</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Month</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Кол-во</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>41</v>
+      </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
+      <c r="C2">
+        <v>247284</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>42</v>
+      </c>
+      <c r="B3">
+        <v>10</v>
+      </c>
+      <c r="C3">
+        <v>157859</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>43</v>
+      </c>
+      <c r="B4">
+        <v>10</v>
+      </c>
+      <c r="C4">
+        <v>189836</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>44</v>
+      </c>
+      <c r="B5">
+        <v>10</v>
+      </c>
+      <c r="C5">
+        <v>171890</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>MEDIUM 800х600х300</v>
+      </c>
+      <c r="B1" t="str">
+        <v>MEDIUM 600х400х400 R-mixed</v>
+      </c>
+      <c r="C1" t="str">
+        <v>MEDIUM 400х300х300 R-mixed</v>
+      </c>
+      <c r="D1" t="str">
+        <v>MEDIUM 400х300х150</v>
+      </c>
+      <c r="E1" t="str">
+        <v>MEDIUM 300*210*100 R-mixed</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Скотч R-mixed</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Скотч цветной</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Стрейч прозрачный</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>10000</v>
+      </c>
+      <c r="B2">
+        <v>23330</v>
+      </c>
+      <c r="C2">
+        <v>10000</v>
+      </c>
+      <c r="D2">
+        <v>15000</v>
+      </c>
+      <c r="E2">
+        <v>10000</v>
+      </c>
+      <c r="F2">
+        <v>10000</v>
+      </c>
+      <c r="G2">
+        <v>1000</v>
+      </c>
+      <c r="H2">
+        <v>10000</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K2"/>
   <sheetData>
     <row r="1">
@@ -7951,88 +8081,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>CW</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Month</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Week 01</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Week 02</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Week 03</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Week 04</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Week 05</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Week 06</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Week 07</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Week 08</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Week 09</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:U34"/>
   <sheetData>

</xml_diff>